<commit_message>
updated inseason ests July 2, 2024
</commit_message>
<xml_diff>
--- a/output/sfsr_inseason_ests_sy24_2024-06-28_11-46-22.xlsx
+++ b/output/sfsr_inseason_ests_sy24_2024-06-28_11-46-22.xlsx
@@ -1,22 +1,84 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\sf_salmon_harvest\output\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37114795-60A7-4248-A74B-A6F2B3118618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="28800" yWindow="0" windowWidth="14400" windowHeight="15750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tag_exp_rel_group" sheetId="1" r:id="rId1"/>
     <sheet name="exp_summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="17">
+  <si>
+    <t>rel_group</t>
+  </si>
+  <si>
+    <t>node</t>
+  </si>
+  <si>
+    <t>n_tags</t>
+  </si>
+  <si>
+    <t>n_tags_exp</t>
+  </si>
+  <si>
+    <t>KNOXB - NOR</t>
+  </si>
+  <si>
+    <t>KRS_D</t>
+  </si>
+  <si>
+    <t>SFG</t>
+  </si>
+  <si>
+    <t>LGR - HOR</t>
+  </si>
+  <si>
+    <t>KRS_U</t>
+  </si>
+  <si>
+    <t>LGR - NOR</t>
+  </si>
+  <si>
+    <t>McCall - Integrated</t>
+  </si>
+  <si>
+    <t>McCall - Segregated</t>
+  </si>
+  <si>
+    <t>SALTRP - NOR</t>
+  </si>
+  <si>
+    <t>SFSRKT - NOR</t>
+  </si>
+  <si>
+    <t>eff_est</t>
+  </si>
+  <si>
+    <t>eff_se</t>
+  </si>
+  <si>
+    <t>tot_est</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -64,13 +126,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -108,7 +178,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -142,6 +212,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -176,9 +247,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -351,42 +423,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>rel_group</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>node</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>n_tags</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>n_tags_exp</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>KNOXB - NOR</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>KRS_D</t>
-        </is>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -395,16 +455,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>KNOXB - NOR</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -413,16 +469,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>LGR - HOR</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>KRS_D</t>
-        </is>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
       </c>
       <c r="C4">
         <v>9</v>
@@ -431,16 +483,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>LGR - HOR</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>KRS_U</t>
-        </is>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
       </c>
       <c r="C5">
         <v>9</v>
@@ -449,16 +497,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>LGR - HOR</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
       </c>
       <c r="C6">
         <v>19</v>
@@ -467,16 +511,12 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>LGR - NOR</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>KRS_D</t>
-        </is>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
       </c>
       <c r="C7">
         <v>40</v>
@@ -485,16 +525,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>LGR - NOR</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>KRS_U</t>
-        </is>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
       </c>
       <c r="C8">
         <v>40</v>
@@ -503,16 +539,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>LGR - NOR</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
       </c>
       <c r="C9">
         <v>130</v>
@@ -521,16 +553,12 @@
         <v>650</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>McCall - Integrated</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>KRS_D</t>
-        </is>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
       </c>
       <c r="C10">
         <v>26</v>
@@ -539,16 +567,12 @@
         <v>203</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>McCall - Integrated</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>KRS_U</t>
-        </is>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
       </c>
       <c r="C11">
         <v>28</v>
@@ -557,16 +581,12 @@
         <v>217</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>McCall - Integrated</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
       </c>
       <c r="C12">
         <v>37</v>
@@ -575,16 +595,12 @@
         <v>280</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>McCall - Segregated</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>KRS_D</t>
-        </is>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
       </c>
       <c r="C13">
         <v>10</v>
@@ -593,16 +609,12 @@
         <v>497</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>McCall - Segregated</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>KRS_U</t>
-        </is>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
       </c>
       <c r="C14">
         <v>11</v>
@@ -611,16 +623,12 @@
         <v>520</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>McCall - Segregated</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
       </c>
       <c r="C15">
         <v>11</v>
@@ -629,16 +637,12 @@
         <v>503</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SALTRP - NOR</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
       </c>
       <c r="C16">
         <v>3</v>
@@ -647,16 +651,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>SFSRKT - NOR</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>KRS_D</t>
-        </is>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
       </c>
       <c r="C17">
         <v>2</v>
@@ -665,16 +665,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>SFSRKT - NOR</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>KRS_U</t>
-        </is>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -683,16 +679,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>SFSRKT - NOR</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
       </c>
       <c r="C19">
         <v>2</v>
@@ -707,57 +699,39 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>rel_group</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>node</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>n_tags</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>n_tags_exp</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>eff_est</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>eff_se</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>tot_est</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>LGR - NOR</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -766,25 +740,21 @@
         <v>650</v>
       </c>
       <c r="E2">
-        <v>0.7736486486486487</v>
+        <v>0.77364864864864868</v>
       </c>
       <c r="F2">
-        <v>0.02038668736303871</v>
+        <v>2.0386687363038711E-2</v>
       </c>
       <c r="G2">
         <v>840</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LGR - NOR</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>KRS_D</t>
-        </is>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
       </c>
       <c r="C3">
         <v>40</v>
@@ -793,25 +763,21 @@
         <v>200</v>
       </c>
       <c r="E3">
-        <v>0.9074074074074074</v>
+        <v>0.90740740740740744</v>
       </c>
       <c r="F3">
-        <v>0.008401920438957476</v>
+        <v>8.4019204389574765E-3</v>
       </c>
       <c r="G3">
         <v>220</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>McCall - Integrated</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
       </c>
       <c r="C4">
         <v>37</v>
@@ -820,25 +786,21 @@
         <v>280</v>
       </c>
       <c r="E4">
-        <v>0.7736486486486487</v>
+        <v>0.77364864864864868</v>
       </c>
       <c r="F4">
-        <v>0.02038668736303871</v>
+        <v>2.0386687363038711E-2</v>
       </c>
       <c r="G4">
         <v>362</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>McCall - Integrated</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>KRS_D</t>
-        </is>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
       </c>
       <c r="C5">
         <v>26</v>
@@ -847,25 +809,21 @@
         <v>203</v>
       </c>
       <c r="E5">
-        <v>0.9074074074074074</v>
+        <v>0.90740740740740744</v>
       </c>
       <c r="F5">
-        <v>0.008401920438957476</v>
+        <v>8.4019204389574765E-3</v>
       </c>
       <c r="G5">
         <v>224</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>McCall - Segregated</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>SFG</t>
-        </is>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
       </c>
       <c r="C6">
         <v>11</v>
@@ -874,25 +832,21 @@
         <v>503</v>
       </c>
       <c r="E6">
-        <v>0.7736486486486487</v>
+        <v>0.77364864864864868</v>
       </c>
       <c r="F6">
-        <v>0.02038668736303871</v>
+        <v>2.0386687363038711E-2</v>
       </c>
       <c r="G6">
         <v>650</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>McCall - Segregated</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>KRS_D</t>
-        </is>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
       </c>
       <c r="C7">
         <v>10</v>
@@ -901,10 +855,10 @@
         <v>497</v>
       </c>
       <c r="E7">
-        <v>0.9074074074074074</v>
+        <v>0.90740740740740744</v>
       </c>
       <c r="F7">
-        <v>0.008401920438957476</v>
+        <v>8.4019204389574765E-3</v>
       </c>
       <c r="G7">
         <v>548</v>

</xml_diff>